<commit_message>
feat: add Arang stage and inventory synergy improvements
</commit_message>
<xml_diff>
--- a/outputs/data-driven-content/balance-template.xlsx
+++ b/outputs/data-driven-content/balance-template.xlsx
@@ -2,16 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Balance" sheetId="1" r:id="R036b345d66604463"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="items" sheetId="2" r:id="Re6ef54f452744c8d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="effects" sheetId="3" r:id="Rfc0f30152798412e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tags" sheetId="4" r:id="Rebeabfd933ba4179"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="loadout" sheetId="5" r:id="Rfb51728561444df2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="encounters" sheetId="6" r:id="R9a94f459e114440c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="rules" sheetId="7" r:id="R93f3d3e51c924e73"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="rewards" sheetId="8" r:id="Rc2cf25b6d19245f1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="routes" sheetId="9" r:id="Ra90fd31238194883"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="events" sheetId="10" r:id="Rec0ca146bad74ca1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Balance" sheetId="1" r:id="R90dc81b424214e9e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="items" sheetId="2" r:id="R05fda92b634f4d23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="effects" sheetId="3" r:id="Rd5f70fa4dd774b77"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tags" sheetId="4" r:id="Rfa443f8ff1a247d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="loadout" sheetId="5" r:id="Rc1a8199c19a34cfe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="encounters" sheetId="6" r:id="Rba5f59c3e78b4886"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="rules" sheetId="7" r:id="R1e142f56abe44d58"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="rewards" sheetId="8" r:id="Rd622ce7bba0c4761"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="routes" sheetId="9" r:id="R6e5d4e95ed26473a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="events" sheetId="10" r:id="Ree93b22460b74415"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="resolutions" sheetId="11" r:id="R171a59f094f44b59"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -55,7 +56,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="7">
+  <x:fills count="8">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -87,6 +88,11 @@
         <x:fgColor rgb="FFFFF0CB"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF29444A"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border>
@@ -100,7 +106,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="28">
+  <x:cellXfs count="31">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <x:extLst>
@@ -184,6 +190,11 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -772,7 +783,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G13" s="19" t="n">
-        <x:f>E13*IF(INDEX(effects!$H$2:$H$2001,MATCH($A13,effects!$A$2:$A$2001,0))="per_adjacent",INDEX(effects!$I$2:$I$2001,MATCH($A13,effects!$A$2:$A$2001,0)),1)</x:f>
+        <x:f>E13*IF(INDEX(effects!$H$2:$H$2001,MATCH($A13,effects!$A$2:$A$2001,0))&lt;&gt;"flat",INDEX(effects!$I$2:$I$2001,MATCH($A13,effects!$A$2:$A$2001,0)),1)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="H13" s="2"/>
@@ -802,7 +813,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G14" s="19" t="n">
-        <x:f>E14*IF(INDEX(effects!$H$2:$H$2001,MATCH($A14,effects!$A$2:$A$2001,0))="per_adjacent",INDEX(effects!$I$2:$I$2001,MATCH($A14,effects!$A$2:$A$2001,0)),1)</x:f>
+        <x:f>E14*IF(INDEX(effects!$H$2:$H$2001,MATCH($A14,effects!$A$2:$A$2001,0))&lt;&gt;"flat",INDEX(effects!$I$2:$I$2001,MATCH($A14,effects!$A$2:$A$2001,0)),1)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="H14" s="2"/>
@@ -832,7 +843,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G15" s="19" t="n">
-        <x:f>E15*IF(INDEX(effects!$H$2:$H$2001,MATCH($A15,effects!$A$2:$A$2001,0))="per_adjacent",INDEX(effects!$I$2:$I$2001,MATCH($A15,effects!$A$2:$A$2001,0)),1)</x:f>
+        <x:f>E15*IF(INDEX(effects!$H$2:$H$2001,MATCH($A15,effects!$A$2:$A$2001,0))&lt;&gt;"flat",INDEX(effects!$I$2:$I$2001,MATCH($A15,effects!$A$2:$A$2001,0)),1)</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="H15" s="2"/>
@@ -862,7 +873,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G16" s="19" t="n">
-        <x:f>E16*IF(INDEX(effects!$H$2:$H$2001,MATCH($A16,effects!$A$2:$A$2001,0))="per_adjacent",INDEX(effects!$I$2:$I$2001,MATCH($A16,effects!$A$2:$A$2001,0)),1)</x:f>
+        <x:f>E16*IF(INDEX(effects!$H$2:$H$2001,MATCH($A16,effects!$A$2:$A$2001,0))&lt;&gt;"flat",INDEX(effects!$I$2:$I$2001,MATCH($A16,effects!$A$2:$A$2001,0)),1)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="H16" s="2"/>
@@ -892,7 +903,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G17" s="19" t="n">
-        <x:f>E17*IF(INDEX(effects!$H$2:$H$2001,MATCH($A17,effects!$A$2:$A$2001,0))="per_adjacent",INDEX(effects!$I$2:$I$2001,MATCH($A17,effects!$A$2:$A$2001,0)),1)</x:f>
+        <x:f>E17*IF(INDEX(effects!$H$2:$H$2001,MATCH($A17,effects!$A$2:$A$2001,0))&lt;&gt;"flat",INDEX(effects!$I$2:$I$2001,MATCH($A17,effects!$A$2:$A$2001,0)),1)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="H17" s="2"/>
@@ -922,7 +933,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G18" s="19" t="n">
-        <x:f>E18*IF(INDEX(effects!$H$2:$H$2001,MATCH($A18,effects!$A$2:$A$2001,0))="per_adjacent",INDEX(effects!$I$2:$I$2001,MATCH($A18,effects!$A$2:$A$2001,0)),1)</x:f>
+        <x:f>E18*IF(INDEX(effects!$H$2:$H$2001,MATCH($A18,effects!$A$2:$A$2001,0))&lt;&gt;"flat",INDEX(effects!$I$2:$I$2001,MATCH($A18,effects!$A$2:$A$2001,0)),1)</x:f>
         <x:v>7</x:v>
       </x:c>
       <x:c r="H18" s="2"/>
@@ -952,7 +963,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G19" s="19" t="n">
-        <x:f>E19*IF(INDEX(effects!$H$2:$H$2001,MATCH($A19,effects!$A$2:$A$2001,0))="per_adjacent",INDEX(effects!$I$2:$I$2001,MATCH($A19,effects!$A$2:$A$2001,0)),1)</x:f>
+        <x:f>E19*IF(INDEX(effects!$H$2:$H$2001,MATCH($A19,effects!$A$2:$A$2001,0))&lt;&gt;"flat",INDEX(effects!$I$2:$I$2001,MATCH($A19,effects!$A$2:$A$2001,0)),1)</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="H19" s="2"/>
@@ -982,7 +993,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G20" s="19" t="n">
-        <x:f>E20*IF(INDEX(effects!$H$2:$H$2001,MATCH($A20,effects!$A$2:$A$2001,0))="per_adjacent",INDEX(effects!$I$2:$I$2001,MATCH($A20,effects!$A$2:$A$2001,0)),1)</x:f>
+        <x:f>E20*IF(INDEX(effects!$H$2:$H$2001,MATCH($A20,effects!$A$2:$A$2001,0))&lt;&gt;"flat",INDEX(effects!$I$2:$I$2001,MATCH($A20,effects!$A$2:$A$2001,0)),1)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="H20" s="2"/>
@@ -1012,7 +1023,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G21" s="19" t="n">
-        <x:f>E21*IF(INDEX(effects!$H$2:$H$2001,MATCH($A21,effects!$A$2:$A$2001,0))="per_adjacent",INDEX(effects!$I$2:$I$2001,MATCH($A21,effects!$A$2:$A$2001,0)),1)</x:f>
+        <x:f>E21*IF(INDEX(effects!$H$2:$H$2001,MATCH($A21,effects!$A$2:$A$2001,0))&lt;&gt;"flat",INDEX(effects!$I$2:$I$2001,MATCH($A21,effects!$A$2:$A$2001,0)),1)</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="H21" s="2"/>
@@ -1042,7 +1053,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G22" s="19" t="n">
-        <x:f>E22*IF(INDEX(effects!$H$2:$H$2001,MATCH($A22,effects!$A$2:$A$2001,0))="per_adjacent",INDEX(effects!$I$2:$I$2001,MATCH($A22,effects!$A$2:$A$2001,0)),1)</x:f>
+        <x:f>E22*IF(INDEX(effects!$H$2:$H$2001,MATCH($A22,effects!$A$2:$A$2001,0))&lt;&gt;"flat",INDEX(effects!$I$2:$I$2001,MATCH($A22,effects!$A$2:$A$2001,0)),1)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="H22" s="2"/>
@@ -1072,7 +1083,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G23" s="19" t="n">
-        <x:f>E23*IF(INDEX(effects!$H$2:$H$2001,MATCH($A23,effects!$A$2:$A$2001,0))="per_adjacent",INDEX(effects!$I$2:$I$2001,MATCH($A23,effects!$A$2:$A$2001,0)),1)</x:f>
+        <x:f>E23*IF(INDEX(effects!$H$2:$H$2001,MATCH($A23,effects!$A$2:$A$2001,0))&lt;&gt;"flat",INDEX(effects!$I$2:$I$2001,MATCH($A23,effects!$A$2:$A$2001,0)),1)</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="H23" s="2"/>
@@ -1102,7 +1113,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G24" s="19" t="n">
-        <x:f>E24*IF(INDEX(effects!$H$2:$H$2001,MATCH($A24,effects!$A$2:$A$2001,0))="per_adjacent",INDEX(effects!$I$2:$I$2001,MATCH($A24,effects!$A$2:$A$2001,0)),1)</x:f>
+        <x:f>E24*IF(INDEX(effects!$H$2:$H$2001,MATCH($A24,effects!$A$2:$A$2001,0))&lt;&gt;"flat",INDEX(effects!$I$2:$I$2001,MATCH($A24,effects!$A$2:$A$2001,0)),1)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="H24" s="2"/>
@@ -1132,7 +1143,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G25" s="19" t="n">
-        <x:f>E25*IF(INDEX(effects!$H$2:$H$2001,MATCH($A25,effects!$A$2:$A$2001,0))="per_adjacent",INDEX(effects!$I$2:$I$2001,MATCH($A25,effects!$A$2:$A$2001,0)),1)</x:f>
+        <x:f>E25*IF(INDEX(effects!$H$2:$H$2001,MATCH($A25,effects!$A$2:$A$2001,0))&lt;&gt;"flat",INDEX(effects!$I$2:$I$2001,MATCH($A25,effects!$A$2:$A$2001,0)),1)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="H25" s="2"/>
@@ -1162,7 +1173,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G26" s="19" t="n">
-        <x:f>E26*IF(INDEX(effects!$H$2:$H$2001,MATCH($A26,effects!$A$2:$A$2001,0))="per_adjacent",INDEX(effects!$I$2:$I$2001,MATCH($A26,effects!$A$2:$A$2001,0)),1)</x:f>
+        <x:f>E26*IF(INDEX(effects!$H$2:$H$2001,MATCH($A26,effects!$A$2:$A$2001,0))&lt;&gt;"flat",INDEX(effects!$I$2:$I$2001,MATCH($A26,effects!$A$2:$A$2001,0)),1)</x:f>
         <x:v>7</x:v>
       </x:c>
       <x:c r="H26" s="2"/>
@@ -1192,7 +1203,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G27" s="19" t="n">
-        <x:f>E27*IF(INDEX(effects!$H$2:$H$2001,MATCH($A27,effects!$A$2:$A$2001,0))="per_adjacent",INDEX(effects!$I$2:$I$2001,MATCH($A27,effects!$A$2:$A$2001,0)),1)</x:f>
+        <x:f>E27*IF(INDEX(effects!$H$2:$H$2001,MATCH($A27,effects!$A$2:$A$2001,0))&lt;&gt;"flat",INDEX(effects!$I$2:$I$2001,MATCH($A27,effects!$A$2:$A$2001,0)),1)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="H27" s="2"/>
@@ -1222,7 +1233,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G28" s="19" t="n">
-        <x:f>E28*IF(INDEX(effects!$H$2:$H$2001,MATCH($A28,effects!$A$2:$A$2001,0))="per_adjacent",INDEX(effects!$I$2:$I$2001,MATCH($A28,effects!$A$2:$A$2001,0)),1)</x:f>
+        <x:f>E28*IF(INDEX(effects!$H$2:$H$2001,MATCH($A28,effects!$A$2:$A$2001,0))&lt;&gt;"flat",INDEX(effects!$I$2:$I$2001,MATCH($A28,effects!$A$2:$A$2001,0)),1)</x:f>
         <x:v>9</x:v>
       </x:c>
       <x:c r="H28" s="2"/>
@@ -1252,7 +1263,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G29" s="19" t="n">
-        <x:f>E29*IF(INDEX(effects!$H$2:$H$2001,MATCH($A29,effects!$A$2:$A$2001,0))="per_adjacent",INDEX(effects!$I$2:$I$2001,MATCH($A29,effects!$A$2:$A$2001,0)),1)</x:f>
+        <x:f>E29*IF(INDEX(effects!$H$2:$H$2001,MATCH($A29,effects!$A$2:$A$2001,0))&lt;&gt;"flat",INDEX(effects!$I$2:$I$2001,MATCH($A29,effects!$A$2:$A$2001,0)),1)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="H29" s="2"/>
@@ -1282,7 +1293,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G30" s="19" t="n">
-        <x:f>E30*IF(INDEX(effects!$H$2:$H$2001,MATCH($A30,effects!$A$2:$A$2001,0))="per_adjacent",INDEX(effects!$I$2:$I$2001,MATCH($A30,effects!$A$2:$A$2001,0)),1)</x:f>
+        <x:f>E30*IF(INDEX(effects!$H$2:$H$2001,MATCH($A30,effects!$A$2:$A$2001,0))&lt;&gt;"flat",INDEX(effects!$I$2:$I$2001,MATCH($A30,effects!$A$2:$A$2001,0)),1)</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="H30" s="2"/>
@@ -1312,7 +1323,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G31" s="19" t="n">
-        <x:f>E31*IF(INDEX(effects!$H$2:$H$2001,MATCH($A31,effects!$A$2:$A$2001,0))="per_adjacent",INDEX(effects!$I$2:$I$2001,MATCH($A31,effects!$A$2:$A$2001,0)),1)</x:f>
+        <x:f>E31*IF(INDEX(effects!$H$2:$H$2001,MATCH($A31,effects!$A$2:$A$2001,0))&lt;&gt;"flat",INDEX(effects!$I$2:$I$2001,MATCH($A31,effects!$A$2:$A$2001,0)),1)</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="H31" s="2"/>
@@ -1427,10 +1438,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="C2" s="27" t="str">
-        <x:v>길가의 동경</x:v>
+        <x:v>대숲의 증거</x:v>
       </x:c>
       <x:c r="D2" s="27" t="str">
-        <x:v>길가에 작은 동경이 놓여 있습니다. 망자가 떠올릴 수 있도록 보따리에 챙길까요?</x:v>
+        <x:v>대숲에서 핏자국이 남은 동경을 찾았다. 진실을 기억할 물건을 챙길까?</x:v>
       </x:c>
       <x:c r="E2" s="27" t="str">
         <x:v>mirror</x:v>
@@ -1442,13 +1453,13 @@
         <x:v>그 자리에 둔다</x:v>
       </x:c>
       <x:c r="H2" s="27" t="str">
-        <x:v>동경을 본 망자가 등불을 떠올리며 숨을 고릅니다. 차사도 잠시 힘을 되찾습니다.</x:v>
+        <x:v>아랑의 원한을 힘으로 가라앉혔다. 동경은 남았지만, 그녀가 전하려던 말은 끝내 듣지 못했다.</x:v>
       </x:c>
       <x:c r="I2" s="27" t="str">
-        <x:v>망자는 동경의 기억을 알아보지 못하지만 차사의 안내를 따라 길을 이어갑니다.</x:v>
+        <x:v>아랑의 원한을 힘으로 가라앉혔다. 그녀의 사연은 여전히 어둠 속에 남아 있다.</x:v>
       </x:c>
       <x:c r="J2" s="27" t="n">
-        <x:v>4</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1464,8 +1475,84 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R69ed61588d094894"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R474ed9faf5db44ad"/>
   </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="40" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="40" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="22" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="28" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="28" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="26" customHeight="1">
+      <x:c r="A1" s="29" t="str">
+        <x:v>id</x:v>
+      </x:c>
+      <x:c r="B1" s="29" t="str">
+        <x:v>event_id</x:v>
+      </x:c>
+      <x:c r="C1" s="29" t="str">
+        <x:v>allow_stash</x:v>
+      </x:c>
+      <x:c r="D1" s="29" t="str">
+        <x:v>message</x:v>
+      </x:c>
+      <x:c r="E1" s="29" t="str">
+        <x:v>result</x:v>
+      </x:c>
+      <x:c r="F1" s="29" t="str">
+        <x:v>button</x:v>
+      </x:c>
+      <x:c r="G1" s="29" t="str">
+        <x:v>unavailable</x:v>
+      </x:c>
+      <x:c r="H1" s="29" t="str">
+        <x:v>completion_title</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="110" customHeight="1">
+      <x:c r="A2" t="str">
+        <x:v>evidence_resolution</x:v>
+      </x:c>
+      <x:c r="B2" t="str">
+        <x:v>lost_keepsake</x:v>
+      </x:c>
+      <x:c r="C2" s="1" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D2" s="30" t="str">
+        <x:v>동경을 보여 주자 아랑이 말을 잇는다.</x:v>
+      </x:c>
+      <x:c r="E2" s="30" t="str">
+        <x:v>아랑은 동경을 알아보고 자신의 억울함을 직접 이야기한다. 차사는 그 말을 명부에 적고, 진실을 전하겠다고 약속한다. 아랑은 고개를 끄덕이며 스스로 길을 나선다.</x:v>
+      </x:c>
+      <x:c r="F2" s="30" t="str">
+        <x:v>동경을 보여 주고 듣는다</x:v>
+      </x:c>
+      <x:c r="G2" s="30" t="str">
+        <x:v>증거를 보따리에 넣으면 아랑의 이야기를 들을 수 있습니다.</x:v>
+      </x:c>
+      <x:c r="H2" s="30" t="str">
+        <x:v>아랑의 밤 · 첫 인도 완료</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="C2:C100">
+      <x:formula1>"TRUE,FALSE"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
 
@@ -1862,10 +1949,10 @@
         <x:v>mirror</x:v>
       </x:c>
       <x:c r="B13" s="9" t="str">
-        <x:v>작은 동경</x:v>
+        <x:v>핏자국이 남은 동경</x:v>
       </x:c>
       <x:c r="C13" s="12" t="str">
-        <x:v>거울에 비친 불빛이 길을 지켜 줍니다.</x:v>
+        <x:v>대숲에서 찾은 동경. 누군가의 마지막 기억이 남아 있다.</x:v>
       </x:c>
       <x:c r="D13" s="9" t="str">
         <x:v>0:0|1:0</x:v>
@@ -1900,7 +1987,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9f45dc38a50a4c53"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9c0590ce6c1a42a0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1983,7 +2070,7 @@
         <x:v>opponent</x:v>
       </x:c>
       <x:c r="E2" s="22" t="n">
-        <x:f>IF(A2="","",ROUND(N2*INDEX(Balance!$B$5:$B$8,MATCH(IF(C2="modify_power",J2,C2),Balance!$A$5:$A$8,0)),0))</x:f>
+        <x:f>IF(A2="","",IF(C2="multiply_power",N2,ROUND(N2*INDEX(Balance!$B$5:$B$8,MATCH(IF(C2="modify_power",J2,C2),Balance!$A$5:$A$8,0)),0)))</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="F2" s="9" t="str"/>
@@ -2020,7 +2107,7 @@
         <x:v>adjacent_items</x:v>
       </x:c>
       <x:c r="E3" s="22" t="n">
-        <x:f>IF(A3="","",ROUND(N3*INDEX(Balance!$B$5:$B$8,MATCH(IF(C3="modify_power",J3,C3),Balance!$A$5:$A$8,0)),0))</x:f>
+        <x:f>IF(A3="","",IF(C3="multiply_power",N3,ROUND(N3*INDEX(Balance!$B$5:$B$8,MATCH(IF(C3="modify_power",J3,C3),Balance!$A$5:$A$8,0)),0)))</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="F3" s="9" t="str">
@@ -2063,7 +2150,7 @@
         <x:v>self</x:v>
       </x:c>
       <x:c r="E4" s="22" t="n">
-        <x:f>IF(A4="","",ROUND(N4*INDEX(Balance!$B$5:$B$8,MATCH(IF(C4="modify_power",J4,C4),Balance!$A$5:$A$8,0)),0))</x:f>
+        <x:f>IF(A4="","",IF(C4="multiply_power",N4,ROUND(N4*INDEX(Balance!$B$5:$B$8,MATCH(IF(C4="modify_power",J4,C4),Balance!$A$5:$A$8,0)),0)))</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="F4" s="9" t="str"/>
@@ -2102,7 +2189,7 @@
         <x:v>self</x:v>
       </x:c>
       <x:c r="E5" s="22" t="n">
-        <x:f>IF(A5="","",ROUND(N5*INDEX(Balance!$B$5:$B$8,MATCH(IF(C5="modify_power",J5,C5),Balance!$A$5:$A$8,0)),0))</x:f>
+        <x:f>IF(A5="","",IF(C5="multiply_power",N5,ROUND(N5*INDEX(Balance!$B$5:$B$8,MATCH(IF(C5="modify_power",J5,C5),Balance!$A$5:$A$8,0)),0)))</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="F5" s="9" t="str"/>
@@ -2139,7 +2226,7 @@
         <x:v>opponent</x:v>
       </x:c>
       <x:c r="E6" s="22" t="n">
-        <x:f>IF(A6="","",ROUND(N6*INDEX(Balance!$B$5:$B$8,MATCH(IF(C6="modify_power",J6,C6),Balance!$A$5:$A$8,0)),0))</x:f>
+        <x:f>IF(A6="","",IF(C6="multiply_power",N6,ROUND(N6*INDEX(Balance!$B$5:$B$8,MATCH(IF(C6="modify_power",J6,C6),Balance!$A$5:$A$8,0)),0)))</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="F6" s="9" t="str"/>
@@ -2176,7 +2263,7 @@
         <x:v>self</x:v>
       </x:c>
       <x:c r="E7" s="22" t="n">
-        <x:f>IF(A7="","",ROUND(N7*INDEX(Balance!$B$5:$B$8,MATCH(IF(C7="modify_power",J7,C7),Balance!$A$5:$A$8,0)),0))</x:f>
+        <x:f>IF(A7="","",IF(C7="multiply_power",N7,ROUND(N7*INDEX(Balance!$B$5:$B$8,MATCH(IF(C7="modify_power",J7,C7),Balance!$A$5:$A$8,0)),0)))</x:f>
         <x:v>7</x:v>
       </x:c>
       <x:c r="F7" s="9" t="str"/>
@@ -2213,7 +2300,7 @@
         <x:v>opponent</x:v>
       </x:c>
       <x:c r="E8" s="22" t="n">
-        <x:f>IF(A8="","",ROUND(N8*INDEX(Balance!$B$5:$B$8,MATCH(IF(C8="modify_power",J8,C8),Balance!$A$5:$A$8,0)),0))</x:f>
+        <x:f>IF(A8="","",IF(C8="multiply_power",N8,ROUND(N8*INDEX(Balance!$B$5:$B$8,MATCH(IF(C8="modify_power",J8,C8),Balance!$A$5:$A$8,0)),0)))</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="F8" s="9" t="str"/>
@@ -2250,7 +2337,7 @@
         <x:v>self</x:v>
       </x:c>
       <x:c r="E9" s="22" t="n">
-        <x:f>IF(A9="","",ROUND(N9*INDEX(Balance!$B$5:$B$8,MATCH(IF(C9="modify_power",J9,C9),Balance!$A$5:$A$8,0)),0))</x:f>
+        <x:f>IF(A9="","",IF(C9="multiply_power",N9,ROUND(N9*INDEX(Balance!$B$5:$B$8,MATCH(IF(C9="modify_power",J9,C9),Balance!$A$5:$A$8,0)),0)))</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="F9" s="9" t="str"/>
@@ -2287,7 +2374,7 @@
         <x:v>opponent</x:v>
       </x:c>
       <x:c r="E10" s="22" t="n">
-        <x:f>IF(A10="","",ROUND(N10*INDEX(Balance!$B$5:$B$8,MATCH(IF(C10="modify_power",J10,C10),Balance!$A$5:$A$8,0)),0))</x:f>
+        <x:f>IF(A10="","",IF(C10="multiply_power",N10,ROUND(N10*INDEX(Balance!$B$5:$B$8,MATCH(IF(C10="modify_power",J10,C10),Balance!$A$5:$A$8,0)),0)))</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="F10" s="9" t="str"/>
@@ -2324,7 +2411,7 @@
         <x:v>self</x:v>
       </x:c>
       <x:c r="E11" s="22" t="n">
-        <x:f>IF(A11="","",ROUND(N11*INDEX(Balance!$B$5:$B$8,MATCH(IF(C11="modify_power",J11,C11),Balance!$A$5:$A$8,0)),0))</x:f>
+        <x:f>IF(A11="","",IF(C11="multiply_power",N11,ROUND(N11*INDEX(Balance!$B$5:$B$8,MATCH(IF(C11="modify_power",J11,C11),Balance!$A$5:$A$8,0)),0)))</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="F11" s="9" t="str"/>
@@ -2361,7 +2448,7 @@
         <x:v>self</x:v>
       </x:c>
       <x:c r="E12" s="22" t="n">
-        <x:f>IF(A12="","",ROUND(N12*INDEX(Balance!$B$5:$B$8,MATCH(IF(C12="modify_power",J12,C12),Balance!$A$5:$A$8,0)),0))</x:f>
+        <x:f>IF(A12="","",IF(C12="multiply_power",N12,ROUND(N12*INDEX(Balance!$B$5:$B$8,MATCH(IF(C12="modify_power",J12,C12),Balance!$A$5:$A$8,0)),0)))</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="F12" s="9" t="str"/>
@@ -2398,7 +2485,7 @@
         <x:v>self</x:v>
       </x:c>
       <x:c r="E13" s="22" t="n">
-        <x:f>IF(A13="","",ROUND(N13*INDEX(Balance!$B$5:$B$8,MATCH(IF(C13="modify_power",J13,C13),Balance!$A$5:$A$8,0)),0))</x:f>
+        <x:f>IF(A13="","",IF(C13="multiply_power",N13,ROUND(N13*INDEX(Balance!$B$5:$B$8,MATCH(IF(C13="modify_power",J13,C13),Balance!$A$5:$A$8,0)),0)))</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="F13" s="9" t="str"/>
@@ -2441,7 +2528,7 @@
         <x:v>opponent</x:v>
       </x:c>
       <x:c r="E14" s="22" t="n">
-        <x:f>IF(A14="","",ROUND(N14*INDEX(Balance!$B$5:$B$8,MATCH(IF(C14="modify_power",J14,C14),Balance!$A$5:$A$8,0)),0))</x:f>
+        <x:f>IF(A14="","",IF(C14="multiply_power",N14,ROUND(N14*INDEX(Balance!$B$5:$B$8,MATCH(IF(C14="modify_power",J14,C14),Balance!$A$5:$A$8,0)),0)))</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="F14" s="9" t="str"/>
@@ -2478,7 +2565,7 @@
         <x:v>opponent</x:v>
       </x:c>
       <x:c r="E15" s="22" t="n">
-        <x:f>IF(A15="","",ROUND(N15*INDEX(Balance!$B$5:$B$8,MATCH(IF(C15="modify_power",J15,C15),Balance!$A$5:$A$8,0)),0))</x:f>
+        <x:f>IF(A15="","",IF(C15="multiply_power",N15,ROUND(N15*INDEX(Balance!$B$5:$B$8,MATCH(IF(C15="modify_power",J15,C15),Balance!$A$5:$A$8,0)),0)))</x:f>
         <x:v>7</x:v>
       </x:c>
       <x:c r="F15" s="9" t="str"/>
@@ -2515,7 +2602,7 @@
         <x:v>self</x:v>
       </x:c>
       <x:c r="E16" s="22" t="n">
-        <x:f>IF(A16="","",ROUND(N16*INDEX(Balance!$B$5:$B$8,MATCH(IF(C16="modify_power",J16,C16),Balance!$A$5:$A$8,0)),0))</x:f>
+        <x:f>IF(A16="","",IF(C16="multiply_power",N16,ROUND(N16*INDEX(Balance!$B$5:$B$8,MATCH(IF(C16="modify_power",J16,C16),Balance!$A$5:$A$8,0)),0)))</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="F16" s="9" t="str"/>
@@ -2552,7 +2639,7 @@
         <x:v>opponent</x:v>
       </x:c>
       <x:c r="E17" s="22" t="n">
-        <x:f>IF(A17="","",ROUND(N17*INDEX(Balance!$B$5:$B$8,MATCH(IF(C17="modify_power",J17,C17),Balance!$A$5:$A$8,0)),0))</x:f>
+        <x:f>IF(A17="","",IF(C17="multiply_power",N17,ROUND(N17*INDEX(Balance!$B$5:$B$8,MATCH(IF(C17="modify_power",J17,C17),Balance!$A$5:$A$8,0)),0)))</x:f>
         <x:v>9</x:v>
       </x:c>
       <x:c r="F17" s="9" t="str"/>
@@ -2589,7 +2676,7 @@
         <x:v>opponent</x:v>
       </x:c>
       <x:c r="E18" s="22" t="n">
-        <x:f>IF(A18="","",ROUND(N18*INDEX(Balance!$B$5:$B$8,MATCH(IF(C18="modify_power",J18,C18),Balance!$A$5:$A$8,0)),0))</x:f>
+        <x:f>IF(A18="","",IF(C18="multiply_power",N18,ROUND(N18*INDEX(Balance!$B$5:$B$8,MATCH(IF(C18="modify_power",J18,C18),Balance!$A$5:$A$8,0)),0)))</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="F18" s="9" t="str"/>
@@ -2626,7 +2713,7 @@
         <x:v>opponent</x:v>
       </x:c>
       <x:c r="E19" s="22" t="n">
-        <x:f>IF(A19="","",ROUND(N19*INDEX(Balance!$B$5:$B$8,MATCH(IF(C19="modify_power",J19,C19),Balance!$A$5:$A$8,0)),0))</x:f>
+        <x:f>IF(A19="","",IF(C19="multiply_power",N19,ROUND(N19*INDEX(Balance!$B$5:$B$8,MATCH(IF(C19="modify_power",J19,C19),Balance!$A$5:$A$8,0)),0)))</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="F19" s="9" t="str"/>
@@ -2663,7 +2750,7 @@
         <x:v>self</x:v>
       </x:c>
       <x:c r="E20" s="22" t="n">
-        <x:f>IF(A20="","",ROUND(N20*INDEX(Balance!$B$5:$B$8,MATCH(IF(C20="modify_power",J20,C20),Balance!$A$5:$A$8,0)),0))</x:f>
+        <x:f>IF(A20="","",IF(C20="multiply_power",N20,ROUND(N20*INDEX(Balance!$B$5:$B$8,MATCH(IF(C20="modify_power",J20,C20),Balance!$A$5:$A$8,0)),0)))</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="F20" s="9" t="str"/>
@@ -2708,17 +2795,17 @@
       <x:formula1>"use,turn_end,damage_taken,modify"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="C2:C2001">
-      <x:formula1>"damage,guard,heal,set_guard,modify_power"</x:formula1>
+      <x:formula1>"damage,guard,heal,set_guard,modify_power,multiply_power"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="D2:D2001">
-      <x:formula1>"self,opponent,adjacent_items"</x:formula1>
+      <x:formula1>"self,opponent,adjacent_items,diagonal_items,neighbor_items"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="whole" operator="between" sqref="E2:E2001">
       <x:formula1>0</x:formula1>
       <x:formula2>100000</x:formula2>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="H2:H2001">
-      <x:formula1>"flat,per_adjacent"</x:formula1>
+      <x:formula1>"flat,per_adjacent,per_diagonal,per_neighbor"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="whole" operator="between" sqref="I2:I2001">
       <x:formula1>1</x:formula1>
@@ -2738,7 +2825,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R94c49937c1cc4d44"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c8feb3948624ebf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2794,7 +2881,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7937145d210644e9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R94a84432ef3648a7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2963,7 +3050,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4f5c417512994f7c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R17446dca08bb457b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3012,7 +3099,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="C2" s="9" t="str">
-        <x:v>길 잃은 그림자</x:v>
+        <x:v>두려움에 사로잡힌 포졸</x:v>
       </x:c>
       <x:c r="D2" s="13" t="n">
         <x:v>18</x:v>
@@ -3033,7 +3120,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C3" s="9" t="str">
-        <x:v>매듭 잡귀</x:v>
+        <x:v>원혼 아랑</x:v>
       </x:c>
       <x:c r="D3" s="13" t="n">
         <x:v>24</x:v>
@@ -3054,7 +3141,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C4" s="9" t="str">
-        <x:v>먹빛 파수꾼</x:v>
+        <x:v>원혼 아랑</x:v>
       </x:c>
       <x:c r="D4" s="13" t="n">
         <x:v>30</x:v>
@@ -3080,7 +3167,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf8afcf0a3c6c4ce7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R225136af98284888"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3169,7 +3256,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc5d56a41c3d14536"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb653f616c7824fc9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3219,7 +3306,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R80da6bd6f8bd4ef4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2b25e120fb0b456a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3257,10 +3344,10 @@
         <x:v>mist_path</x:v>
       </x:c>
       <x:c r="B2" s="9" t="str">
-        <x:v>안개 고갯길</x:v>
+        <x:v>대숲을 따라간다</x:v>
       </x:c>
       <x:c r="C2" s="12" t="str">
-        <x:v>매듭 잡귀를 먼저 만나고 먹빛 파수꾼에게 향합니다.</x:v>
+        <x:v>대숲에서 아랑을 만납니다. 첫 행동은 방어이며 체력이 낮습니다.</x:v>
       </x:c>
       <x:c r="D2" s="12" t="str">
         <x:v>gate_1|gate_2|gate_3</x:v>
@@ -3274,10 +3361,10 @@
         <x:v>moon_path</x:v>
       </x:c>
       <x:c r="B3" s="9" t="str">
-        <x:v>달그늘 샛길</x:v>
+        <x:v>연못을 지나간다</x:v>
       </x:c>
       <x:c r="C3" s="12" t="str">
-        <x:v>먹빛 파수꾼을 먼저 넘어 매듭 잡귀에게 향합니다.</x:v>
+        <x:v>연못을 지나 아랑을 만납니다. 첫 행동은 공격이며 체력이 높습니다.</x:v>
       </x:c>
       <x:c r="D3" s="12" t="str">
         <x:v>gate_1|gate_3|gate_2</x:v>
@@ -3289,7 +3376,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra482ea476a26425e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbe0771475ce74a49"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
improving crossroads and intent visualization
</commit_message>
<xml_diff>
--- a/outputs/data-driven-content/balance-template.xlsx
+++ b/outputs/data-driven-content/balance-template.xlsx
@@ -2,17 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Balance" sheetId="1" r:id="R90dc81b424214e9e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="items" sheetId="2" r:id="R05fda92b634f4d23"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="effects" sheetId="3" r:id="Rd5f70fa4dd774b77"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tags" sheetId="4" r:id="Rfa443f8ff1a247d3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="loadout" sheetId="5" r:id="Rc1a8199c19a34cfe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="encounters" sheetId="6" r:id="Rba5f59c3e78b4886"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="rules" sheetId="7" r:id="R1e142f56abe44d58"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="rewards" sheetId="8" r:id="Rd622ce7bba0c4761"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="routes" sheetId="9" r:id="R6e5d4e95ed26473a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="events" sheetId="10" r:id="Ree93b22460b74415"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="resolutions" sheetId="11" r:id="R171a59f094f44b59"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Balance" sheetId="1" r:id="Rc5973266ba104921"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="items" sheetId="2" r:id="R61c6d1918b1e4697"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="effects" sheetId="3" r:id="Rb9d4a2c52712429d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tags" sheetId="4" r:id="Rf9cac5aa2ab840d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="loadout" sheetId="5" r:id="Rc987a1a6879f43b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="encounters" sheetId="6" r:id="R895dc9976b28429d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="rules" sheetId="7" r:id="R7d7ead5d209b4d41"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="rewards" sheetId="8" r:id="R41ce6719652d4fa3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="routes" sheetId="9" r:id="Rd50c818621614c0c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="events" sheetId="10" r:id="Raa3f8ace57ad4548"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="resolutions" sheetId="11" r:id="R31dd7022fae547bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="hazards" sheetId="12" r:id="R79195c194587477a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -56,7 +57,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="8">
+  <x:fills count="9">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -93,6 +94,11 @@
         <x:fgColor rgb="FF29444A"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF29444A"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border>
@@ -106,7 +112,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="31">
+  <x:cellXfs count="33">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <x:extLst>
@@ -196,6 +202,8 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -640,7 +648,7 @@
       </x:c>
       <x:c r="E5" s="19" t="n">
         <x:f>COUNTA(effects!A2:A2001)</x:f>
-        <x:v>19</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="F5" s="19" t="n">
         <x:f>COUNTA(encounters!A2:A2001)</x:f>
@@ -1329,23 +1337,63 @@
       <x:c r="H31" s="2"/>
     </x:row>
     <x:row r="32" ht="26" customHeight="1">
-      <x:c r="A32" s="2"/>
-      <x:c r="B32" s="2"/>
-      <x:c r="C32" s="2"/>
-      <x:c r="D32" s="2"/>
-      <x:c r="E32" s="2"/>
-      <x:c r="F32" s="2"/>
-      <x:c r="G32" s="2"/>
+      <x:c r="A32" s="2" t="str">
+        <x:v>jade_diagonal_factor</x:v>
+      </x:c>
+      <x:c r="B32" s="2" t="str">
+        <x:f>INDEX(effects!$C$2:$C$2001,MATCH($A32,effects!$A$2:$A$2001,0))</x:f>
+        <x:v>multiply_power</x:v>
+      </x:c>
+      <x:c r="C32" s="2" t="str">
+        <x:f>INDEX(effects!$B$2:$B$2001,MATCH($A32,effects!$A$2:$A$2001,0))</x:f>
+        <x:v>modify</x:v>
+      </x:c>
+      <x:c r="D32" s="19" t="n">
+        <x:f>INDEX(effects!$N$2:$N$2001,MATCH($A32,effects!$A$2:$A$2001,0))</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E32" s="19" t="n">
+        <x:f>INDEX(effects!$E$2:$E$2001,MATCH($A32,effects!$A$2:$A$2001,0))</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F32" s="19" t="n">
+        <x:f>E32-D32</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G32" s="19" t="n">
+        <x:f>E32*IF(INDEX(effects!$H$2:$H$2001,MATCH($A32,effects!$A$2:$A$2001,0))&lt;&gt;"flat",INDEX(effects!$I$2:$I$2001,MATCH($A32,effects!$A$2:$A$2001,0)),1)</x:f>
+        <x:v>2</x:v>
+      </x:c>
       <x:c r="H32" s="2"/>
     </x:row>
     <x:row r="33" ht="26" customHeight="1">
-      <x:c r="A33" s="2"/>
-      <x:c r="B33" s="2"/>
-      <x:c r="C33" s="2"/>
-      <x:c r="D33" s="2"/>
-      <x:c r="E33" s="2"/>
-      <x:c r="F33" s="2"/>
-      <x:c r="G33" s="2"/>
+      <x:c r="A33" s="2" t="str">
+        <x:v>arang_pain_reaction</x:v>
+      </x:c>
+      <x:c r="B33" s="2" t="str">
+        <x:f>INDEX(effects!$C$2:$C$2001,MATCH($A33,effects!$A$2:$A$2001,0))</x:f>
+        <x:v>damage</x:v>
+      </x:c>
+      <x:c r="C33" s="2" t="str">
+        <x:f>INDEX(effects!$B$2:$B$2001,MATCH($A33,effects!$A$2:$A$2001,0))</x:f>
+        <x:v>damage_taken</x:v>
+      </x:c>
+      <x:c r="D33" s="19" t="n">
+        <x:f>INDEX(effects!$N$2:$N$2001,MATCH($A33,effects!$A$2:$A$2001,0))</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E33" s="19" t="n">
+        <x:f>INDEX(effects!$E$2:$E$2001,MATCH($A33,effects!$A$2:$A$2001,0))</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F33" s="19" t="n">
+        <x:f>E33-D33</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G33" s="19" t="n">
+        <x:f>E33*IF(INDEX(effects!$H$2:$H$2001,MATCH($A33,effects!$A$2:$A$2001,0))&lt;&gt;"flat",INDEX(effects!$I$2:$I$2001,MATCH($A33,effects!$A$2:$A$2001,0)),1)</x:f>
+        <x:v>2</x:v>
+      </x:c>
       <x:c r="H33" s="2"/>
     </x:row>
     <x:row r="34" ht="26" customHeight="1">
@@ -1438,25 +1486,25 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="C2" s="27" t="str">
-        <x:v>대숲의 증거</x:v>
+        <x:v>Evidence in the Grove</x:v>
       </x:c>
       <x:c r="D2" s="27" t="str">
-        <x:v>대숲에서 핏자국이 남은 동경을 찾았다. 진실을 기억할 물건을 챙길까?</x:v>
+        <x:v>A bloodstained mirror lies in the bamboo grove. Will you keep it as evidence?</x:v>
       </x:c>
       <x:c r="E2" s="27" t="str">
         <x:v>mirror</x:v>
       </x:c>
       <x:c r="F2" s="27" t="str">
-        <x:v>동경을 챙긴다</x:v>
+        <x:v>Take the mirror</x:v>
       </x:c>
       <x:c r="G2" s="27" t="str">
-        <x:v>그 자리에 둔다</x:v>
+        <x:v>Leave it</x:v>
       </x:c>
       <x:c r="H2" s="27" t="str">
-        <x:v>아랑의 원한을 힘으로 가라앉혔다. 동경은 남았지만, 그녀가 전하려던 말은 끝내 듣지 못했다.</x:v>
+        <x:v>You subdued Arang by force. The mirror remains, but her story was left untold.</x:v>
       </x:c>
       <x:c r="I2" s="27" t="str">
-        <x:v>아랑의 원한을 힘으로 가라앉혔다. 그녀의 사연은 여전히 어둠 속에 남아 있다.</x:v>
+        <x:v>You subdued Arang by force. Her story remains untold.</x:v>
       </x:c>
       <x:c r="J2" s="27" t="n">
         <x:v>0</x:v>
@@ -1475,7 +1523,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R474ed9faf5db44ad"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2dd6e5ae76194fd3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1531,19 +1579,19 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D2" s="30" t="str">
-        <x:v>동경을 보여 주자 아랑이 말을 잇는다.</x:v>
+        <x:v>Arang recognizes the mirror and begins to speak.</x:v>
       </x:c>
       <x:c r="E2" s="30" t="str">
-        <x:v>아랑은 동경을 알아보고 자신의 억울함을 직접 이야기한다. 차사는 그 말을 명부에 적고, 진실을 전하겠다고 약속한다. 아랑은 고개를 끄덕이며 스스로 길을 나선다.</x:v>
+        <x:v>Arang recognizes the mirror and tells you what happened. You record her words and promise to reveal the truth. She nods and sets out on her own.</x:v>
       </x:c>
       <x:c r="F2" s="30" t="str">
-        <x:v>동경을 보여 주고 듣는다</x:v>
+        <x:v>Show the mirror and listen</x:v>
       </x:c>
       <x:c r="G2" s="30" t="str">
-        <x:v>증거를 보따리에 넣으면 아랑의 이야기를 들을 수 있습니다.</x:v>
+        <x:v>Place the evidence in your bag to hear Arang's story.</x:v>
       </x:c>
       <x:c r="H2" s="30" t="str">
-        <x:v>아랑의 밤 · 첫 인도 완료</x:v>
+        <x:v>Arang's Night · First Delivery Complete</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1552,6 +1600,70 @@
       <x:formula1>"TRUE,FALSE"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="20" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="20" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="35" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="20" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="20" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="20" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="58" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="26" customHeight="1">
+      <x:c r="A1" s="32" t="str">
+        <x:v>id</x:v>
+      </x:c>
+      <x:c r="B1" s="32" t="str">
+        <x:v>step</x:v>
+      </x:c>
+      <x:c r="C1" s="32" t="str">
+        <x:v>cells</x:v>
+      </x:c>
+      <x:c r="D1" s="32" t="str">
+        <x:v>required_tags</x:v>
+      </x:c>
+      <x:c r="E1" s="32" t="str">
+        <x:v>cost_increase</x:v>
+      </x:c>
+      <x:c r="F1" s="32" t="str">
+        <x:v>label</x:v>
+      </x:c>
+      <x:c r="G1" s="32" t="str">
+        <x:v>description</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="55" customHeight="1">
+      <x:c r="A2" t="str">
+        <x:v>edge_frost</x:v>
+      </x:c>
+      <x:c r="B2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C2" t="str">
+        <x:v>0:0|1:0|2:0|3:0|4:0</x:v>
+      </x:c>
+      <x:c r="D2" t="str">
+        <x:v>weapon</x:v>
+      </x:c>
+      <x:c r="E2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F2" t="str">
+        <x:v>Spirit's Chill</x:v>
+      </x:c>
+      <x:c r="G2" s="30" t="str">
+        <x:v>Cold has settled on the bag. Rotate or move a weapon to avoid it.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
@@ -1609,10 +1721,10 @@
         <x:v>sword</x:v>
       </x:c>
       <x:c r="B2" s="9" t="str">
-        <x:v>낡은 사인검</x:v>
+        <x:v>Sain Sword</x:v>
       </x:c>
       <x:c r="C2" s="12" t="str">
-        <x:v>상하좌우의 물건에 따라 위력이 달라지는 오래된 검.</x:v>
+        <x:v>An old sword whose power changes with nearby items.</x:v>
       </x:c>
       <x:c r="D2" s="9" t="str">
         <x:v>0:0|0:1|0:2</x:v>
@@ -1641,10 +1753,10 @@
         <x:v>seal</x:v>
       </x:c>
       <x:c r="B3" s="9" t="str">
-        <x:v>봉인부</x:v>
+        <x:v>Sealing Talisman</x:v>
       </x:c>
       <x:c r="C3" s="12" t="str">
-        <x:v>인접한 무기를 강화합니다. 대각선은 인접하지 않습니다.</x:v>
+        <x:v>Strengthens weapons directly adjacent to it.</x:v>
       </x:c>
       <x:c r="D3" s="9" t="str">
         <x:v>0:0</x:v>
@@ -1673,10 +1785,10 @@
         <x:v>lantern</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>혼백등</x:v>
+        <x:v>Soul Lantern</x:v>
       </x:c>
       <x:c r="C4" s="12" t="str">
-        <x:v>망자의 물건이 어두운 길을 비춥니다.</x:v>
+        <x:v>Lights the way for the belongings of the dead.</x:v>
       </x:c>
       <x:c r="D4" s="9" t="str">
         <x:v>0:0|0:1</x:v>
@@ -1705,10 +1817,10 @@
         <x:v>ring</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>옥가락지</x:v>
+        <x:v>Jade Ring</x:v>
       </x:c>
       <x:c r="C5" s="12" t="str">
-        <x:v>돌려주지 못한 마지막 약속을 담은 유품.</x:v>
+        <x:v>Doubles the attack power of weapons diagonally adjacent.</x:v>
       </x:c>
       <x:c r="D5" s="9" t="str">
         <x:v>0:0</x:v>
@@ -1728,17 +1840,19 @@
       <x:c r="I5" s="9" t="str">
         <x:v>ring</x:v>
       </x:c>
-      <x:c r="J5" s="12" t="str"/>
+      <x:c r="J5" s="12" t="str">
+        <x:v>jade_diagonal_factor</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="48" customHeight="1">
       <x:c r="A6" s="9" t="str">
         <x:v>hat</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>낡은 갓</x:v>
+        <x:v>Worn Gat</x:v>
       </x:c>
       <x:c r="C6" s="12" t="str">
-        <x:v>다음 적 행동까지 피해를 막습니다. 넓은 챙만큼 보따리 자리도 많이 필요합니다.</x:v>
+        <x:v>Blocks damage until the next enemy action. Its wide brim takes up space.</x:v>
       </x:c>
       <x:c r="D6" s="9" t="str">
         <x:v>0:0|1:0|0:1|1:1</x:v>
@@ -1765,10 +1879,10 @@
         <x:v>bell</x:v>
       </x:c>
       <x:c r="B7" s="9" t="str">
-        <x:v>길잡이 방울</x:v>
+        <x:v>Guide Bell</x:v>
       </x:c>
       <x:c r="C7" s="12" t="str">
-        <x:v>작은 공간으로 추가 공격을 확보합니다. 무기 태그가 없어 봉인부 강화는 받지 않습니다.</x:v>
+        <x:v>A compact extra attack. It has no weapon tag and cannot receive talisman bonuses.</x:v>
       </x:c>
       <x:c r="D7" s="9" t="str">
         <x:v>0:0</x:v>
@@ -1795,10 +1909,10 @@
         <x:v>yakgwa</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>작은 약과</x:v>
+        <x:v>Small Yakgwa</x:v>
       </x:c>
       <x:c r="C8" s="12" t="str">
-        <x:v>한 번 먹으면 사라져 공간이 비어납니다. 배치를 되돌려도 되살릴 수 없습니다.</x:v>
+        <x:v>A one-use honey pastry. Once eaten, its space is freed permanently.</x:v>
       </x:c>
       <x:c r="D8" s="9" t="str">
         <x:v>0:0</x:v>
@@ -1825,10 +1939,10 @@
         <x:v>rope</x:v>
       </x:c>
       <x:c r="B9" s="9" t="str">
-        <x:v>오라</x:v>
+        <x:v>Binding Rope</x:v>
       </x:c>
       <x:c r="C9" s="12" t="str">
-        <x:v>꺾인 형태의 무기. 회전해 틈에 넣고 인접 보너스를 활용하세요.</x:v>
+        <x:v>A bent weapon. Rotate it to fit gaps and use adjacency bonuses.</x:v>
       </x:c>
       <x:c r="D9" s="9" t="str">
         <x:v>0:0|0:1|1:1</x:v>
@@ -1857,10 +1971,10 @@
         <x:v>sandals</x:v>
       </x:c>
       <x:c r="B10" s="9" t="str">
-        <x:v>짚신</x:v>
+        <x:v>Straw Shoes</x:v>
       </x:c>
       <x:c r="C10" s="12" t="str">
-        <x:v>갓보다 작은 방어 도구. 남은 공간으로 다른 물건을 챙길 수 있습니다.</x:v>
+        <x:v>A compact defense tool that leaves more room for other items.</x:v>
       </x:c>
       <x:c r="D10" s="9" t="str">
         <x:v>0:0|0:1</x:v>
@@ -1887,10 +2001,10 @@
         <x:v>order</x:v>
       </x:c>
       <x:c r="B11" s="9" t="str">
-        <x:v>적패지</x:v>
+        <x:v>Reaper Writ</x:v>
       </x:c>
       <x:c r="C11" s="12" t="str">
-        <x:v>인도 명령을 담은 문서. 큰 힘을 쓰는 만큼 기력을 아껴야 합니다. 능력은 게임용 창작입니다.</x:v>
+        <x:v>A delivery order with a powerful attack that requires careful energy management.</x:v>
       </x:c>
       <x:c r="D11" s="9" t="str">
         <x:v>0:0|0:1</x:v>
@@ -1917,10 +2031,10 @@
         <x:v>coin</x:v>
       </x:c>
       <x:c r="B12" s="9" t="str">
-        <x:v>남겨진 엽전</x:v>
+        <x:v>Forgotten Coin</x:v>
       </x:c>
       <x:c r="C12" s="12" t="str">
-        <x:v>기력을 쓰지 않고 작은 방어를 얻는 유품.</x:v>
+        <x:v>A keepsake that gives a little defense without spending energy.</x:v>
       </x:c>
       <x:c r="D12" s="9" t="str">
         <x:v>0:0</x:v>
@@ -1949,10 +2063,10 @@
         <x:v>mirror</x:v>
       </x:c>
       <x:c r="B13" s="9" t="str">
-        <x:v>핏자국이 남은 동경</x:v>
+        <x:v>Bloodstained Mirror</x:v>
       </x:c>
       <x:c r="C13" s="12" t="str">
-        <x:v>대숲에서 찾은 동경. 누군가의 마지막 기억이 남아 있다.</x:v>
+        <x:v>A mirror found in the bamboo grove, holding someone's last memories.</x:v>
       </x:c>
       <x:c r="D13" s="9" t="str">
         <x:v>0:0|1:0</x:v>
@@ -1987,7 +2101,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9c0590ce6c1a42a0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R61ef7176e45d4744"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2774,20 +2888,82 @@
       </x:c>
     </x:row>
     <x:row r="21">
-      <x:c r="A21"/>
-      <x:c r="B21"/>
-      <x:c r="C21"/>
-      <x:c r="D21"/>
-      <x:c r="E21"/>
-      <x:c r="F21"/>
-      <x:c r="G21"/>
-      <x:c r="H21"/>
-      <x:c r="I21"/>
-      <x:c r="J21"/>
-      <x:c r="K21"/>
-      <x:c r="L21"/>
-      <x:c r="M21"/>
-      <x:c r="N21"/>
+      <x:c r="A21" s="9" t="str">
+        <x:v>jade_diagonal_factor</x:v>
+      </x:c>
+      <x:c r="B21" s="9" t="str">
+        <x:v>modify</x:v>
+      </x:c>
+      <x:c r="C21" s="9" t="str">
+        <x:v>multiply_power</x:v>
+      </x:c>
+      <x:c r="D21" s="9" t="str">
+        <x:v>diagonal_items</x:v>
+      </x:c>
+      <x:c r="E21" s="22" t="n">
+        <x:f>IF(A21="","",IF(C21="multiply_power",N21,ROUND(N21*INDEX(Balance!$B$5:$B$8,MATCH(IF(C21="modify_power",J21,C21),Balance!$A$5:$A$8,0)),0)))</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F21" s="9" t="str">
+        <x:v>weapon</x:v>
+      </x:c>
+      <x:c r="G21" s="9" t="str"/>
+      <x:c r="H21" s="9" t="str">
+        <x:v>flat</x:v>
+      </x:c>
+      <x:c r="I21" s="13" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J21" s="9" t="str">
+        <x:v>damage</x:v>
+      </x:c>
+      <x:c r="K21" s="9" t="str"/>
+      <x:c r="L21" s="13" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M21" s="13" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N21" s="9" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="9" t="str">
+        <x:v>arang_pain_reaction</x:v>
+      </x:c>
+      <x:c r="B22" s="9" t="str">
+        <x:v>damage_taken</x:v>
+      </x:c>
+      <x:c r="C22" s="9" t="str">
+        <x:v>damage</x:v>
+      </x:c>
+      <x:c r="D22" s="9" t="str">
+        <x:v>opponent</x:v>
+      </x:c>
+      <x:c r="E22" s="22" t="n">
+        <x:f>IF(A22="","",IF(C22="multiply_power",N22,ROUND(N22*INDEX(Balance!$B$5:$B$8,MATCH(IF(C22="modify_power",J22,C22),Balance!$A$5:$A$8,0)),0)))</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F22" s="9" t="str"/>
+      <x:c r="G22" s="9" t="str"/>
+      <x:c r="H22" s="9" t="str">
+        <x:v>flat</x:v>
+      </x:c>
+      <x:c r="I22" s="13" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J22" s="9" t="str"/>
+      <x:c r="K22" s="9" t="str"/>
+      <x:c r="L22" s="13" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M22" s="13" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N22" s="9" t="n">
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="9">
@@ -2825,7 +3001,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c8feb3948624ebf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9f5c48de5d384499"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2851,7 +3027,7 @@
         <x:v>weapon</x:v>
       </x:c>
       <x:c r="B2" s="9" t="str">
-        <x:v>무기</x:v>
+        <x:v>Weapon</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="28" customHeight="1">
@@ -2859,7 +3035,7 @@
         <x:v>keepsake</x:v>
       </x:c>
       <x:c r="B3" s="9" t="str">
-        <x:v>유품</x:v>
+        <x:v>Keepsake</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="28" customHeight="1">
@@ -2867,7 +3043,7 @@
         <x:v>lantern</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>등</x:v>
+        <x:v>Lantern</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="28" customHeight="1">
@@ -2875,13 +3051,13 @@
         <x:v>talisman</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>talisman</x:v>
+        <x:v>Talisman</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R94a84432ef3648a7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rafe35dde51be4f8f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3050,7 +3226,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R17446dca08bb457b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3e4a0df19199465a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3099,7 +3275,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="C2" s="9" t="str">
-        <x:v>두려움에 사로잡힌 포졸</x:v>
+        <x:v>Terrified Guard</x:v>
       </x:c>
       <x:c r="D2" s="13" t="n">
         <x:v>18</x:v>
@@ -3120,10 +3296,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C3" s="9" t="str">
-        <x:v>원혼 아랑</x:v>
+        <x:v>Arang, Restless Spirit</x:v>
       </x:c>
       <x:c r="D3" s="13" t="n">
-        <x:v>24</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="E3" s="12" t="str">
         <x:v>encounter_2_intent_1|encounter_2_intent_2</x:v>
@@ -3141,15 +3317,17 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C4" s="9" t="str">
-        <x:v>원혼 아랑</x:v>
+        <x:v>Arang, Restless Spirit</x:v>
       </x:c>
       <x:c r="D4" s="13" t="n">
-        <x:v>30</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="E4" s="12" t="str">
         <x:v>encounter_3_intent_1|encounter_3_intent_2|encounter_3_intent_3</x:v>
       </x:c>
-      <x:c r="F4" s="12" t="str"/>
+      <x:c r="F4" s="12" t="str">
+        <x:v>arang_pain_reaction</x:v>
+      </x:c>
       <x:c r="G4" s="9" t="str">
         <x:v>spirit_3</x:v>
       </x:c>
@@ -3167,7 +3345,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R225136af98284888"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R151a8a4aa2c54635"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3256,7 +3434,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb653f616c7824fc9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R65783f6cda0c4229"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3289,7 +3467,7 @@
         <x:v>gate_1</x:v>
       </x:c>
       <x:c r="C2" s="12" t="str">
-        <x:v>rope|sandals|mirror</x:v>
+        <x:v>rope|sandals|order</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="48" customHeight="1">
@@ -3306,7 +3484,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2b25e120fb0b456a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d546c32b6d2441c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3344,10 +3522,10 @@
         <x:v>mist_path</x:v>
       </x:c>
       <x:c r="B2" s="9" t="str">
-        <x:v>대숲을 따라간다</x:v>
+        <x:v>Follow the Bamboo Grove</x:v>
       </x:c>
       <x:c r="C2" s="12" t="str">
-        <x:v>대숲에서 아랑을 만납니다. 첫 행동은 방어이며 체력이 낮습니다.</x:v>
+        <x:v>Meet Arang in the grove. Her first move is defense.</x:v>
       </x:c>
       <x:c r="D2" s="12" t="str">
         <x:v>gate_1|gate_2|gate_3</x:v>
@@ -3361,10 +3539,10 @@
         <x:v>moon_path</x:v>
       </x:c>
       <x:c r="B3" s="9" t="str">
-        <x:v>연못을 지나간다</x:v>
+        <x:v>Pass the Moonlit Pond</x:v>
       </x:c>
       <x:c r="C3" s="12" t="str">
-        <x:v>연못을 지나 아랑을 만납니다. 첫 행동은 공격이며 체력이 높습니다.</x:v>
+        <x:v>Meet Arang by the pond. Her first move is an attack.</x:v>
       </x:c>
       <x:c r="D3" s="12" t="str">
         <x:v>gate_1|gate_3|gate_2</x:v>
@@ -3376,7 +3554,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbe0771475ce74a49"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfaa6d9d9a0174d41"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>